<commit_message>
V2 - Connected MySQL DB and created UI
</commit_message>
<xml_diff>
--- a/MoodMate_Analysis.xlsx
+++ b/MoodMate_Analysis.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -501,238 +501,22 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Disappointed</t>
+          <t>Satisfied</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Redmi Note 10</t>
+          <t>Redmi 12 5G</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Redmi 12 5G</t>
+          <t>Redmi 13C 5G</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>If you're considering an exchange, you can also explore these similar-priced phones.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Redmi Note 9 Pro</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Full display not working in all application.</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>3.0 out of 5 stars</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Others</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Quite good</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Disappointed</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Redmi Note 11</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Redmi 13</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>I understand you're a bit disappointed, so you might consider Redmi Note 11 or Redmi 13 as optional options.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Redmi Note 9 Pro Max</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Not worth for the money</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>2.0 out of 5 stars</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Others</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>worst product from MI. I am a hardcore fan of MI. But this one really disappointing.</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Disappointed</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Redmi Note 12</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Redmi Note 10 Pro</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>I'm sorry you're disappointed; you might consider the Redmi Note 12 or Redmi Note 10 Pro.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Redmi 9</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Fabulous!</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>4.0 out of 5 stars</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Display</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Pros:
-notch display
-Dual camera
-Face unlock
-4000 mah battery
-Cons:
-Some of the apps donot work in full screen mode.
-No Front flash
-Great product to purchase finally and its value for money.I got this phone for 10,500 and thanks to Xiaomi.</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Satisfied</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Redmi 14C</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>Redmi 12</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>I’m glad you’re happy with your Redmi 9; if you’d like to explore a larger, higher‑refresh display and bigger battery, you might consider the Redmi 14C or Redmi 12.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Redmi 9 Power</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Fantastic</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>4.0 out of 5 stars</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Camera</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Front camera is poor rest things are good</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Satisfied</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Redmi 13C 5G</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Redmi 13C</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>If you'd like a better front camera, you might try the Redmi 13C 5G or Redmi 13C.</t>
+          <t>I understand you’d like a larger screen—these two models offer bigger displays while staying close to your budget.</t>
         </is>
       </c>
     </row>

</xml_diff>